<commit_message>
add 2 role user
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="users" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -49,7 +50,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -412,10 +413,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="161.109375" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -458,15 +463,69 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>scrypt:32768:8:1$qajnxX75get14j3T$998d257ea704785df7123d1bfbdca09878adf26a13eb429e92b6a718108faf8e257e58b1b75346b67f48237b45a44238adb9f064810dfb525d70311690ff6f51</t>
+          <t>scrypt:32768:8:1$YvC835gbNk6xd9sy$87f7fc4a0d8cb59f5c542e89ac603d838d252c68f2fd6326e5430d83d72f5b14adcc944f6c64a095376656b274a90e103817db17fdaa2980e7adc22b19b98fcd</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>10000002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Developer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$Awop6owzwcxDsIry$805a02a3c6baf4e1c45ebe4c4d06f59aa33587657e95c48bb43bccf759596cae189f7631a78c0ec91d23916d0326a201baf66c041176ce49644cdabeb2e3e5db</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>developer</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>90000001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Tsel</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>scrypt:32768:8:1$WkcVTPGf6uD3Q0Gn$17e9982d99fd4b48e8e984e1e63b746bc225d8bafeee9b692bcf140e57bd1bdab03f3348e0cfd1c0c74c4ec4f7335bc7c8adb91aa825a51b939131281cba3e4f</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>viewer</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>ALL</t>
         </is>

</xml_diff>